<commit_message>
update: import template with 26 congregations
</commit_message>
<xml_diff>
--- a/plantilla_importar_publicadores.xlsx
+++ b/plantilla_importar_publicadores.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Publicadores" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Ayuda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Congregaciones" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -511,12 +512,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>María</t>
+          <t>Maria</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>González</t>
+          <t>Gonzalez</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -570,7 +571,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Apellido casada (opcional)</t>
+          <t>Apellido casada</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -580,12 +581,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Email (opcional)</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Teléfono</t>
+          <t>Telefono</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -595,22 +596,22 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Email del cónyuge en PPAM (opcional)</t>
+          <t>Email conyuge PPAM</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>ID de la congregación (ver hoja Ayuda)</t>
+          <t>ID congregacion (ver hoja Congregaciones)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Designaciones JSON (opcional)</t>
+          <t>Designaciones JSON</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Notas (opcional)</t>
+          <t>Notas</t>
         </is>
       </c>
     </row>
@@ -640,7 +641,7 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>DESCRIPCIÓN</t>
+          <t>DESCRIPCION</t>
         </is>
       </c>
     </row>
@@ -700,7 +701,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Email para inicio de sesión. Si se deja vacío no se crea usuario.</t>
+          <t>Email para inicio de sesion. Vacio = no se crea usuario.</t>
         </is>
       </c>
     </row>
@@ -712,7 +713,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Teléfono en formato libre.</t>
+          <t>Telefono en formato libre.</t>
         </is>
       </c>
     </row>
@@ -724,7 +725,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SOLTERO, CASADO, DIVORCIADO, SEPARADO, o VIUDO.</t>
+          <t>SOLTERO, CASADO, DIVORCIADO, SEPARADO, VIUDO.</t>
         </is>
       </c>
     </row>
@@ -736,7 +737,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Email del cónyuge si ya está en PPAM. Si no, dejar vacío.</t>
+          <t>Email del conyuge si ya esta en PPAM. Vacio si no.</t>
         </is>
       </c>
     </row>
@@ -748,7 +749,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ID de la congregación. Debe existir en el sistema (ver hoja Congregaciones).</t>
+          <t>ID de la congregacion. Ver hoja Congregaciones.</t>
         </is>
       </c>
     </row>
@@ -760,7 +761,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JSON: ["ANCIANO","PRECURSOR_REGULAR","SIERVO_MINISTERIAL","MISIONERO","PRECURSOR_ESPECIAL","FAMILIA_BETEL","PUBLICADOR"]</t>
+          <t>JSON: ["ANCIANO","PRECURSOR_REGULAR","SIERVO_MINISTERIAL",...]</t>
         </is>
       </c>
     </row>
@@ -773,6 +774,348 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>Notas adicionales (opcional).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1f63a7fc-6940-4999-9bf5-728d502620f0</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Alto Mirador - San Antonio</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>b3ef5456-4122-41a5-9486-ab55d5ee0306</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Barrancas - San Antonio</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>b9b15417-66ad-43c7-b306-c51f1332572b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Barrio Oriente - Melipilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>49cb3f18-f908-493d-89eb-677fb21cb637</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Brisas de Culipran - Melipilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>64ec34cf-5292-4bf0-ae6b-f9f4b0feda94</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Centenario - San Antonio</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4927859c-5c7b-4168-b516-db90a9364bfe</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Central - Melipilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>c54e0fae-d37b-4240-8589-1ac18cd43ae5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Costa Azul - Cartagena</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>3e758822-2970-4dff-816c-cf8e885881e6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Costanera - El Quisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>029db583-9714-40f9-8e2d-4898f735372a</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Criollo Haitiano Melipilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>636ecf00-fb62-417d-b7ba-1624785abcea</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Criollo Haitiano San Antonio</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>c034fade-08e7-417d-b35d-47149cdb686e</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>El Canelo - Algarrobo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>cad483fd-00f1-49cf-905b-24b2754ca75a</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>El Tabo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>88f76fe2-8382-48fa-be53-9d5b7d7edf25</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>El Totoral - El Quisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>63f475ad-a6cb-48a4-bdf5-34ad86170f37</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>El Tranque - Llolleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>05af16f6-e994-4543-80b8-e824bbc90963</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Isla Negra</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>6d939a38-7654-411f-9501-6578dbc91ad9</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Litoral - Cartagena</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>38db7727-4738-487e-a804-243e66c41b45</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Lo Abarca - Cartagena</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>186a1977-9cb2-4e5c-860d-3515b139cd2e</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Lomas - Llolleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10e45fca-0c7e-4ad6-944e-eb37606606e4</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Los Boldos - Bollenar</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>258ad838-9d8b-4d5b-bef8-70861140e7ec</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Mirasol - Algarrobo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>44ff763e-a1e2-4e88-be2e-41817eea1c7c</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Pabellon - Melipilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>bcd9e619-f7ac-4555-8bc6-b0fbbdde115d</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Pomaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>104b70da-463c-4343-b79b-79510f75b061</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Riberas del Maipo - Santo Domingo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>095fcf42-e128-49f1-9b2a-a618204918e2</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Sol Poniente - Melipilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>b4380cad-4ec6-47ae-b7ad-52867e824c7f</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Valle de Mallarauco - Bollenar</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>32c7c1a1-cc9a-4b90-b153-7a27164c5493</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Villa Alhue</t>
         </is>
       </c>
     </row>

</xml_diff>